<commit_message>
feat: Add PDF Highlighter Enhancement Summary & Comparison Script
- Introduced a new script to analyze and summarize improvements made to the PDF highlighter.
- The script loads performance results from a JSON file and presents a detailed summary of enhancements.
- Major improvements categorized into visual system, text matching, quote extraction, performance optimization, error handling, analytics, and configuration.
- Added a comparison section highlighting differences between the old and new highlighter functionalities.
- Included technical innovations and expected benefits of the enhancements.
- Provided usage examples for processing studies with various options.
</commit_message>
<xml_diff>
--- a/Data/20250729_location choie_unit of analysis.xlsx
+++ b/Data/20250729_location choie_unit of analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ugentbe-my.sharepoint.com/personal/kuralarasan_kumar_ugent_be/Documents/My Projects/Grafitti Project/Urban_Foraging_Archive/Articles_drafts/2024 Snatching/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4466DD8E-7FE9-49A7-B7B6-7E855009FAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{4466DD8E-7FE9-49A7-B7B6-7E855009FAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{55FB22E3-4DD8-4477-A763-70118CF8AF5E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{1E22BB9B-89AF-4CFF-A417-35485B719593}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{1E22BB9B-89AF-4CFF-A417-35485B719593}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
     <author>tc={D365743D-D521-4E47-A224-B0820E5F4BEE}</author>
   </authors>
   <commentList>
-    <comment ref="D32" authorId="0" shapeId="0" xr:uid="{D365743D-D521-4E47-A224-B0820E5F4BEE}">
+    <comment ref="D51" authorId="0" shapeId="0" xr:uid="{D365743D-D521-4E47-A224-B0820E5F4BEE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1042,7 +1042,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="D32" dT="2025-07-02T12:34:51.88" personId="{9A7316DD-6F33-4137-8F70-BB862D6D0A49}" id="{D365743D-D521-4E47-A224-B0820E5F4BEE}">
+  <threadedComment ref="D51" dT="2025-07-02T12:34:51.88" personId="{9A7316DD-6F33-4137-8F70-BB862D6D0A49}" id="{D365743D-D521-4E47-A224-B0820E5F4BEE}">
     <text>Ask Wim about the area of the street segment</text>
   </threadedComment>
 </ThreadedComments>
@@ -1051,21 +1051,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EE16F5C-9A23-431F-BBFB-BA5A34AA640B}">
   <dimension ref="A1:J70"/>
-  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="69.6640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="34.44140625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="17.88671875" style="8" customWidth="1"/>
-    <col min="5" max="5" width="9.109375" style="8"/>
-    <col min="6" max="7" width="9.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="23.88671875" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="23.88671875" style="8" customWidth="1"/>
+    <col min="1" max="1" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="69.7109375" style="8" customWidth="1"/>
+    <col min="3" max="3" width="34.42578125" style="8" customWidth="1"/>
+    <col min="4" max="4" width="17.85546875" style="8" customWidth="1"/>
+    <col min="5" max="5" width="9.140625" style="8"/>
+    <col min="6" max="7" width="9.28515625" style="8" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" style="8" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="23.85546875" style="8" customWidth="1"/>
     <col min="10" max="10" width="84" style="7" customWidth="1"/>
-    <col min="11" max="16384" width="9.109375" style="8"/>
+    <col min="11" max="16384" width="9.140625" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1097,207 +1097,207 @@
         <v>124</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A2" s="14">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>8</v>
+        <v>94</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>9</v>
+        <v>95</v>
       </c>
       <c r="D2" s="14">
-        <v>19680</v>
+        <v>136</v>
       </c>
       <c r="E2" s="14" t="s">
         <v>155</v>
       </c>
       <c r="F2" s="14">
-        <v>24594</v>
+        <v>503589</v>
       </c>
       <c r="G2" s="14">
-        <v>12938</v>
+        <v>4308</v>
       </c>
       <c r="H2" s="14" t="s">
-        <v>10</v>
+        <v>96</v>
       </c>
       <c r="I2" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J2" s="12"/>
     </row>
-    <row r="3" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="14">
-        <v>2</v>
+        <v>34</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>12</v>
+        <v>83</v>
       </c>
       <c r="D3" s="14">
-        <v>19680</v>
+        <v>2.96</v>
       </c>
       <c r="E3" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3" s="14">
+        <v>4000</v>
+      </c>
+      <c r="G3" s="14">
+        <v>7179</v>
+      </c>
+      <c r="H3" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J3" s="12"/>
+    </row>
+    <row r="4" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="14">
+        <v>9</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" s="14">
+        <v>2.96</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F4" s="14">
+        <v>142</v>
+      </c>
+      <c r="G4" s="14">
+        <v>12639</v>
+      </c>
+      <c r="H4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I4" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J4" s="12"/>
+    </row>
+    <row r="5" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="14">
+        <v>30</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="D5" s="14">
+        <v>40000</v>
+      </c>
+      <c r="E5" s="14" t="s">
         <v>155</v>
       </c>
-      <c r="F3" s="14">
-        <v>24594</v>
-      </c>
-      <c r="G3" s="14">
-        <v>12938</v>
-      </c>
-      <c r="H3" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="I3" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J3" s="12"/>
-    </row>
-    <row r="4" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A4" s="14">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="s">
+      <c r="F5" s="14">
+        <v>4.5579999999999998</v>
+      </c>
+      <c r="G5" s="14">
+        <v>165</v>
+      </c>
+      <c r="H5" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="I5" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J5" s="12"/>
+    </row>
+    <row r="6" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A6" s="14">
+        <v>16</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="D6" s="14">
+        <v>1.62</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F6" s="14">
+        <v>1971</v>
+      </c>
+      <c r="G6" s="14">
+        <v>4358</v>
+      </c>
+      <c r="H6" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I6" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J6" s="12"/>
+    </row>
+    <row r="7" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="14">
+        <v>15</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="D7" s="14">
+        <v>1.62</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F7" s="14">
+        <v>1973</v>
+      </c>
+      <c r="G7" s="14">
+        <v>1262</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J7" s="12"/>
+    </row>
+    <row r="8" spans="1:10" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="14">
         <v>13</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="14">
-        <v>6.7</v>
-      </c>
-      <c r="E4" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F4" s="14">
-        <v>291</v>
-      </c>
-      <c r="G4" s="14">
-        <v>1761</v>
-      </c>
-      <c r="H4" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J4" s="12"/>
-    </row>
-    <row r="5" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A5" s="14">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D5" s="14">
-        <v>8.48</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F5" s="14">
-        <v>158</v>
-      </c>
-      <c r="G5" s="14">
-        <v>889</v>
-      </c>
-      <c r="H5" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="I5" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J5" s="12"/>
-    </row>
-    <row r="6" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
-      <c r="A6" s="14">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" s="14">
-        <v>8.48</v>
-      </c>
-      <c r="E6" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F6" s="14">
-        <v>158</v>
-      </c>
-      <c r="G6" s="14">
-        <v>2844</v>
-      </c>
-      <c r="H6" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="I6" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J6" s="12"/>
-    </row>
-    <row r="7" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A7" s="14">
-        <v>6</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="14">
-        <v>2.96</v>
-      </c>
-      <c r="E7" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F7" s="14">
-        <v>142</v>
-      </c>
-      <c r="G7" s="14">
-        <v>12639</v>
-      </c>
-      <c r="H7" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="I7" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J7" s="12"/>
-    </row>
-    <row r="8" spans="1:10" ht="62.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="14">
-        <v>7</v>
-      </c>
       <c r="B8" s="3" t="s">
-        <v>24</v>
+        <v>36</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="D8" s="14">
-        <v>2.96</v>
+        <v>1.68</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F8" s="14">
-        <v>142</v>
+        <v>76</v>
       </c>
       <c r="G8" s="14">
-        <v>3037</v>
+        <v>13088</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>23</v>
@@ -1309,15 +1309,15 @@
         <v>154</v>
       </c>
     </row>
-    <row r="9" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="14">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D9" s="14">
         <v>2.96</v>
@@ -1329,7 +1329,7 @@
         <v>142</v>
       </c>
       <c r="G9" s="14">
-        <v>19420</v>
+        <v>12639</v>
       </c>
       <c r="H9" s="14" t="s">
         <v>23</v>
@@ -1339,147 +1339,147 @@
       </c>
       <c r="J9" s="12"/>
     </row>
-    <row r="10" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A10" s="14">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>28</v>
+        <v>62</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="D10" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F10" s="14">
+        <v>89</v>
+      </c>
+      <c r="G10" s="14">
+        <v>548</v>
+      </c>
+      <c r="H10" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J10" s="12"/>
+    </row>
+    <row r="11" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A11" s="14">
+        <v>4</v>
+      </c>
+      <c r="B11" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="14">
+        <v>8.48</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F11" s="14">
+        <v>158</v>
+      </c>
+      <c r="G11" s="14">
+        <v>889</v>
+      </c>
+      <c r="H11" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J11" s="12"/>
+    </row>
+    <row r="12" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A12" s="14">
+        <v>12</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D12" s="14">
+        <v>2.04</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F12" s="14">
+        <v>131</v>
+      </c>
+      <c r="G12" s="14">
+        <v>398</v>
+      </c>
+      <c r="H12" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J12" s="12"/>
+    </row>
+    <row r="13" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A13" s="14">
+        <v>10</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D13" s="14">
+        <v>2.74</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F13" s="14">
+        <v>2643</v>
+      </c>
+      <c r="G13" s="14">
+        <v>3860</v>
+      </c>
+      <c r="H13" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J13" s="12"/>
+    </row>
+    <row r="14" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A14" s="14">
+        <v>7</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="14">
         <v>2.96</v>
       </c>
-      <c r="E10" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F10" s="14">
+      <c r="E14" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F14" s="14">
         <v>142</v>
       </c>
-      <c r="G10" s="14">
-        <v>12639</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="I10" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J10" s="12"/>
-    </row>
-    <row r="11" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A11" s="14">
-        <v>10</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="D11" s="14">
-        <v>2.74</v>
-      </c>
-      <c r="E11" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F11" s="14">
-        <v>2643</v>
-      </c>
-      <c r="G11" s="14">
-        <v>3860</v>
-      </c>
-      <c r="H11" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I11" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J11" s="12"/>
-    </row>
-    <row r="12" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
-      <c r="A12" s="14">
-        <v>11</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D12" s="14">
-        <v>2.1800000000000002</v>
-      </c>
-      <c r="E12" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F12" s="14">
-        <v>201</v>
-      </c>
-      <c r="G12" s="14">
-        <v>1573</v>
-      </c>
-      <c r="H12" s="14" t="s">
-        <v>129</v>
-      </c>
-      <c r="I12" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J12" s="12"/>
-    </row>
-    <row r="13" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A13" s="14">
-        <v>12</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D13" s="14">
-        <v>2.04</v>
-      </c>
-      <c r="E13" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F13" s="14">
-        <v>131</v>
-      </c>
-      <c r="G13" s="14">
-        <v>398</v>
-      </c>
-      <c r="H13" s="14" t="s">
-        <v>128</v>
-      </c>
-      <c r="I13" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J13" s="12"/>
-    </row>
-    <row r="14" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A14" s="14">
-        <v>13</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D14" s="14">
-        <v>1.68</v>
-      </c>
-      <c r="E14" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F14" s="14">
-        <v>76</v>
-      </c>
       <c r="G14" s="14">
-        <v>13088</v>
+        <v>3037</v>
       </c>
       <c r="H14" s="14" t="s">
         <v>23</v>
@@ -1489,45 +1489,45 @@
       </c>
       <c r="J14" s="12"/>
     </row>
-    <row r="15" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A15" s="14">
+        <v>24</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="E15" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F15" s="14">
+        <v>89</v>
+      </c>
+      <c r="G15" s="14">
+        <v>1174</v>
+      </c>
+      <c r="H15" s="14" t="s">
+        <v>47</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J15" s="12"/>
+    </row>
+    <row r="16" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A16" s="14">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B16" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>39</v>
-      </c>
-      <c r="D15" s="14">
-        <v>1.62</v>
-      </c>
-      <c r="E15" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F15" s="14">
-        <v>1616</v>
-      </c>
-      <c r="G15" s="14">
-        <v>3436</v>
-      </c>
-      <c r="H15" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="I15" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J15" s="12"/>
-    </row>
-    <row r="16" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A16" s="14">
-        <v>15</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>42</v>
       </c>
       <c r="D16" s="14">
         <v>1.62</v>
@@ -1536,80 +1536,80 @@
         <v>156</v>
       </c>
       <c r="F16" s="14">
-        <v>1973</v>
+        <v>1616</v>
       </c>
       <c r="G16" s="14">
-        <v>1262</v>
+        <v>3436</v>
       </c>
       <c r="H16" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J16" s="12"/>
+    </row>
+    <row r="17" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A17" s="14">
+        <v>48</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="12">
+        <v>3.2000000000000001E-2</v>
+      </c>
+      <c r="E17" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F17" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="G17" s="12">
+        <v>425</v>
+      </c>
+      <c r="H17" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J17" s="12"/>
+    </row>
+    <row r="18" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A18" s="14">
+        <v>49</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="D18" s="12">
+        <v>0.95799999999999996</v>
+      </c>
+      <c r="E18" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F18" s="12">
+        <v>1652</v>
+      </c>
+      <c r="G18" s="12">
+        <v>1972</v>
+      </c>
+      <c r="H18" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="I16" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J16" s="12"/>
-    </row>
-    <row r="17" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A17" s="14">
-        <v>16</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="14">
-        <v>1.62</v>
-      </c>
-      <c r="E17" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F17" s="14">
-        <v>1971</v>
-      </c>
-      <c r="G17" s="14">
-        <v>4358</v>
-      </c>
-      <c r="H17" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="I17" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J17" s="12"/>
-    </row>
-    <row r="18" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
-      <c r="A18" s="14">
-        <v>17</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" s="14">
-        <v>1.62</v>
-      </c>
-      <c r="E18" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F18" s="14">
-        <v>1971</v>
-      </c>
-      <c r="G18" s="14">
-        <v>7860</v>
-      </c>
-      <c r="H18" s="14" t="s">
-        <v>47</v>
-      </c>
       <c r="I18" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J18" s="12"/>
     </row>
-    <row r="19" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A19" s="14">
         <v>18</v>
       </c>
@@ -1639,30 +1639,30 @@
       </c>
       <c r="J19" s="12"/>
     </row>
-    <row r="20" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A20" s="14">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="D20" s="14">
-        <v>1.41</v>
+        <v>1.62</v>
       </c>
       <c r="E20" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F20" s="14">
-        <v>2153</v>
+        <v>1971</v>
       </c>
       <c r="G20" s="14">
-        <v>38120</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>130</v>
+        <v>7860</v>
+      </c>
+      <c r="H20" s="14" t="s">
+        <v>47</v>
       </c>
       <c r="I20" s="14" t="s">
         <v>126</v>
@@ -1671,57 +1671,57 @@
         <v>131</v>
       </c>
     </row>
-    <row r="21" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A21" s="14">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>52</v>
+        <v>11</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="D21" s="14">
-        <v>0.79</v>
+        <v>19680</v>
       </c>
       <c r="E21" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F21" s="14">
-        <v>193</v>
+        <v>24594</v>
       </c>
       <c r="G21" s="14">
-        <v>679</v>
+        <v>12938</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>132</v>
+        <v>10</v>
       </c>
       <c r="I21" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J21" s="12"/>
     </row>
-    <row r="22" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A22" s="14">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="D22" s="14">
-        <v>2.63</v>
+        <v>0.65</v>
       </c>
       <c r="E22" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F22" s="14">
-        <v>12821</v>
+        <v>89</v>
       </c>
       <c r="G22" s="14">
-        <v>140</v>
+        <v>26000</v>
       </c>
       <c r="H22" s="14" t="s">
         <v>47</v>
@@ -1731,330 +1731,330 @@
       </c>
       <c r="J22" s="12"/>
     </row>
-    <row r="23" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A23" s="14">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>56</v>
+        <v>86</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>57</v>
+        <v>87</v>
       </c>
       <c r="D23" s="14">
-        <v>2.63</v>
+        <v>2.96</v>
       </c>
       <c r="E23" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F23" s="14">
-        <v>71</v>
+        <v>4006</v>
       </c>
       <c r="G23" s="14">
-        <v>13305</v>
+        <v>276</v>
       </c>
       <c r="H23" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J23" s="12"/>
+    </row>
+    <row r="24" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A24" s="14">
+        <v>50</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="D24" s="12">
+        <v>1.2</v>
+      </c>
+      <c r="E24" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F24" s="12">
+        <v>2153</v>
+      </c>
+      <c r="G24" s="13">
+        <v>38120</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J24" s="12"/>
+    </row>
+    <row r="25" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A25" s="14">
+        <v>8</v>
+      </c>
+      <c r="B25" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D25" s="14">
+        <v>2.96</v>
+      </c>
+      <c r="E25" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F25" s="14">
+        <v>142</v>
+      </c>
+      <c r="G25" s="14">
+        <v>19420</v>
+      </c>
+      <c r="H25" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J25" s="12"/>
+    </row>
+    <row r="26" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A26" s="14">
+        <v>3</v>
+      </c>
+      <c r="B26" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D26" s="14">
+        <v>6.7</v>
+      </c>
+      <c r="E26" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F26" s="14">
+        <v>291</v>
+      </c>
+      <c r="G26" s="14">
+        <v>1761</v>
+      </c>
+      <c r="H26" s="14" t="s">
+        <v>15</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J26" s="12"/>
+    </row>
+    <row r="27" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A27" s="14">
+        <v>1</v>
+      </c>
+      <c r="B27" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="14">
+        <v>19680</v>
+      </c>
+      <c r="E27" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F27" s="14">
+        <v>24594</v>
+      </c>
+      <c r="G27" s="14">
+        <v>12938</v>
+      </c>
+      <c r="H27" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J27" s="12"/>
+    </row>
+    <row r="28" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
+      <c r="A28" s="14">
+        <v>46</v>
+      </c>
+      <c r="B28" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="D28" s="5">
+        <v>844.91</v>
+      </c>
+      <c r="E28" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F28" s="18">
+        <v>2233</v>
+      </c>
+      <c r="G28" s="18">
+        <v>12655</v>
+      </c>
+      <c r="H28" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J28" s="12"/>
+    </row>
+    <row r="29" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A29" s="14">
+        <v>23</v>
+      </c>
+      <c r="B29" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="14">
+        <v>0.65</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F29" s="14">
+        <v>89</v>
+      </c>
+      <c r="G29" s="14">
+        <v>548</v>
+      </c>
+      <c r="H29" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J23" s="12"/>
-    </row>
-    <row r="24" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A24" s="14">
-        <v>23</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C24" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="D24" s="14">
-        <v>0.65</v>
-      </c>
-      <c r="E24" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F24" s="14">
-        <v>89</v>
-      </c>
-      <c r="G24" s="14">
-        <v>548</v>
-      </c>
-      <c r="H24" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="I24" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J24" s="12"/>
-    </row>
-    <row r="25" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
-      <c r="A25" s="14">
-        <v>24</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D25" s="14">
-        <v>0.65</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F25" s="14">
-        <v>89</v>
-      </c>
-      <c r="G25" s="14">
-        <v>1174</v>
-      </c>
-      <c r="H25" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="I25" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J25" s="12"/>
-    </row>
-    <row r="26" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
-      <c r="A26" s="14">
-        <v>25</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C26" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D26" s="14">
-        <v>0.65</v>
-      </c>
-      <c r="E26" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F26" s="14">
-        <v>89</v>
-      </c>
-      <c r="G26" s="14">
-        <v>548</v>
-      </c>
-      <c r="H26" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="I26" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J26" s="12"/>
-    </row>
-    <row r="27" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A27" s="14">
-        <v>26</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C27" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D27" s="14">
-        <v>0.65</v>
-      </c>
-      <c r="E27" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F27" s="14">
-        <v>89</v>
-      </c>
-      <c r="G27" s="14">
-        <v>26000</v>
-      </c>
-      <c r="H27" s="14" t="s">
-        <v>47</v>
-      </c>
-      <c r="I27" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J27" s="12"/>
-    </row>
-    <row r="28" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A28" s="14">
+      <c r="I29" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J29" s="12"/>
+    </row>
+    <row r="30" spans="1:10" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A30" s="14">
+        <v>45</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="D30" s="17">
+        <v>2.81</v>
+      </c>
+      <c r="E30" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F30" s="12">
+        <v>1636</v>
+      </c>
+      <c r="G30" s="12">
+        <v>1540</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="J30" s="12"/>
+    </row>
+    <row r="31" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="A31" s="14">
         <v>27</v>
       </c>
-      <c r="B28" s="3" t="s">
+      <c r="B31" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C31" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="D28" s="14">
+      <c r="D31" s="14">
         <v>0.51</v>
       </c>
-      <c r="E28" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F28" s="14">
+      <c r="E31" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F31" s="14">
         <v>1687</v>
       </c>
-      <c r="G28" s="14">
+      <c r="G31" s="14">
         <v>3337</v>
       </c>
-      <c r="H28" s="14" t="s">
+      <c r="H31" s="14" t="s">
         <v>133</v>
       </c>
-      <c r="I28" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J28" s="12"/>
-    </row>
-    <row r="29" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A29" s="14">
-        <v>28</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="D29" s="14">
-        <v>0.44</v>
-      </c>
-      <c r="E29" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F29" s="14">
-        <v>616</v>
-      </c>
-      <c r="G29" s="14">
-        <v>1105</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="I29" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J29" s="12"/>
-    </row>
-    <row r="30" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A30" s="14">
-        <v>29</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C30" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="D30" s="14">
-        <v>25000</v>
-      </c>
-      <c r="E30" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="F30" s="14">
-        <v>1134</v>
-      </c>
-      <c r="G30" s="14">
-        <v>369</v>
-      </c>
-      <c r="H30" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="I30" s="14" t="s">
-        <v>126</v>
-      </c>
-      <c r="J30" s="12"/>
-    </row>
-    <row r="31" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A31" s="14">
-        <v>30</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C31" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="14">
-        <v>40000</v>
-      </c>
-      <c r="E31" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="F31" s="14">
-        <v>4.5579999999999998</v>
-      </c>
-      <c r="G31" s="14">
-        <v>165</v>
-      </c>
-      <c r="H31" s="14" t="s">
-        <v>71</v>
-      </c>
       <c r="I31" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J31" s="12"/>
     </row>
-    <row r="32" spans="1:10" s="11" customFormat="1" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:10" s="11" customFormat="1" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A32" s="14">
-        <v>31</v>
-      </c>
-      <c r="B32" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C32" s="15" t="s">
-        <v>75</v>
-      </c>
-      <c r="D32" s="16">
-        <v>1545</v>
+        <v>11</v>
+      </c>
+      <c r="B32" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C32" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D32" s="14">
+        <v>2.1800000000000002</v>
       </c>
       <c r="E32" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="F32" s="16">
-        <v>262</v>
-      </c>
-      <c r="G32" s="16">
-        <v>50</v>
-      </c>
-      <c r="H32" s="16" t="s">
-        <v>76</v>
+        <v>156</v>
+      </c>
+      <c r="F32" s="14">
+        <v>201</v>
+      </c>
+      <c r="G32" s="14">
+        <v>1573</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>129</v>
       </c>
       <c r="I32" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J32" s="20"/>
     </row>
-    <row r="33" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A33" s="14">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>77</v>
+        <v>52</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>78</v>
+        <v>53</v>
       </c>
       <c r="D33" s="14">
-        <v>0.7</v>
+        <v>0.79</v>
       </c>
       <c r="E33" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F33" s="14">
-        <v>844</v>
+        <v>193</v>
       </c>
       <c r="G33" s="14">
-        <v>12872</v>
+        <v>679</v>
       </c>
       <c r="H33" s="14" t="s">
-        <v>79</v>
+        <v>132</v>
       </c>
       <c r="I33" s="14" t="s">
         <v>126</v>
@@ -2063,30 +2063,30 @@
         <v>135</v>
       </c>
     </row>
-    <row r="34" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A34" s="14">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="D34" s="14">
-        <v>0.88</v>
+        <v>2.96</v>
       </c>
       <c r="E34" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F34" s="14">
-        <v>334</v>
+        <v>23984</v>
       </c>
       <c r="G34" s="14">
-        <v>5182</v>
+        <v>1871</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>137</v>
+        <v>23</v>
       </c>
       <c r="I34" s="14" t="s">
         <v>126</v>
@@ -2095,30 +2095,30 @@
         <v>136</v>
       </c>
     </row>
-    <row r="35" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A35" s="14">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B35" s="3" t="s">
-        <v>82</v>
+        <v>67</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>83</v>
+        <v>68</v>
       </c>
       <c r="D35" s="14">
-        <v>2.96</v>
+        <v>0.44</v>
       </c>
       <c r="E35" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F35" s="14">
-        <v>4000</v>
+        <v>616</v>
       </c>
       <c r="G35" s="14">
-        <v>7179</v>
-      </c>
-      <c r="H35" s="14" t="s">
-        <v>23</v>
+        <v>1105</v>
+      </c>
+      <c r="H35" s="3" t="s">
+        <v>134</v>
       </c>
       <c r="I35" s="14" t="s">
         <v>126</v>
@@ -2127,30 +2127,30 @@
         <v>138</v>
       </c>
     </row>
-    <row r="36" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A36" s="14">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>85</v>
+        <v>100</v>
       </c>
       <c r="D36" s="14">
-        <v>2.96</v>
+        <v>0.15</v>
       </c>
       <c r="E36" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F36" s="14">
-        <v>23984</v>
+        <v>890</v>
       </c>
       <c r="G36" s="14">
-        <v>1871</v>
+        <v>150</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>23</v>
+        <v>101</v>
       </c>
       <c r="I36" s="14" t="s">
         <v>126</v>
@@ -2159,30 +2159,30 @@
         <v>138</v>
       </c>
     </row>
-    <row r="37" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A37" s="14">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="B37" s="3" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="D37" s="14">
-        <v>2.96</v>
+        <v>1.41</v>
       </c>
       <c r="E37" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F37" s="14">
-        <v>4006</v>
+        <v>2153</v>
       </c>
       <c r="G37" s="14">
-        <v>276</v>
-      </c>
-      <c r="H37" s="14" t="s">
-        <v>23</v>
+        <v>38120</v>
+      </c>
+      <c r="H37" s="3" t="s">
+        <v>130</v>
       </c>
       <c r="I37" s="14" t="s">
         <v>126</v>
@@ -2191,30 +2191,30 @@
         <v>138</v>
       </c>
     </row>
-    <row r="38" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A38" s="14">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B38" s="3" t="s">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="C38" s="5" t="s">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="D38" s="14">
-        <v>2.8400000000000002E-2</v>
+        <v>0.88</v>
       </c>
       <c r="E38" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F38" s="14">
-        <v>5286</v>
+        <v>334</v>
       </c>
       <c r="G38" s="14">
-        <v>459</v>
+        <v>5182</v>
       </c>
       <c r="H38" s="14" t="s">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="I38" s="14" t="s">
         <v>126</v>
@@ -2223,30 +2223,30 @@
         <v>139</v>
       </c>
     </row>
-    <row r="39" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A39" s="14">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D39" s="14">
-        <v>0.33</v>
+        <v>142.27000000000001</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F39" s="14">
-        <v>4.7649999999999997</v>
+        <v>300</v>
       </c>
       <c r="G39" s="14">
-        <v>2299</v>
+        <v>2911</v>
       </c>
       <c r="H39" s="14" t="s">
-        <v>141</v>
+        <v>96</v>
       </c>
       <c r="I39" s="14" t="s">
         <v>126</v>
@@ -2255,30 +2255,30 @@
         <v>140</v>
       </c>
     </row>
-    <row r="40" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A40" s="14">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B40" s="3" t="s">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="C40" s="5" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="D40" s="14">
-        <v>0.2</v>
+        <v>2.63</v>
       </c>
       <c r="E40" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F40" s="14">
-        <v>198</v>
+        <v>71</v>
       </c>
       <c r="G40" s="14">
-        <v>721</v>
+        <v>13305</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>141</v>
+        <v>47</v>
       </c>
       <c r="I40" s="14" t="s">
         <v>126</v>
@@ -2287,90 +2287,90 @@
         <v>142</v>
       </c>
     </row>
-    <row r="41" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A41" s="14">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C41" s="5" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="D41" s="14">
-        <v>136</v>
+        <v>2.8400000000000002E-2</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="F41" s="14">
-        <v>503589</v>
+        <v>5286</v>
       </c>
       <c r="G41" s="14">
-        <v>4308</v>
+        <v>459</v>
       </c>
       <c r="H41" s="14" t="s">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="I41" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J41" s="12"/>
     </row>
-    <row r="42" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A42" s="14">
-        <v>41</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>97</v>
+        <v>47</v>
+      </c>
+      <c r="B42" s="5" t="s">
+        <v>149</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="D42" s="14">
-        <v>142.27000000000001</v>
+        <v>123</v>
+      </c>
+      <c r="D42" s="5">
+        <v>0.37</v>
       </c>
       <c r="E42" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="F42" s="14">
-        <v>300</v>
-      </c>
-      <c r="G42" s="14">
-        <v>2911</v>
-      </c>
-      <c r="H42" s="14" t="s">
-        <v>96</v>
+        <v>156</v>
+      </c>
+      <c r="F42" s="5">
+        <v>653</v>
+      </c>
+      <c r="G42" s="18">
+        <v>6249</v>
+      </c>
+      <c r="H42" s="5" t="s">
+        <v>109</v>
       </c>
       <c r="I42" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J42" s="12"/>
     </row>
-    <row r="43" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A43" s="14">
-        <v>42</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D43" s="14">
-        <v>0.15</v>
+        <v>51</v>
+      </c>
+      <c r="B43" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D43" s="12">
+        <v>6.2E-2</v>
       </c>
       <c r="E43" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F43" s="14">
-        <v>890</v>
-      </c>
-      <c r="G43" s="14">
-        <v>150</v>
-      </c>
-      <c r="H43" s="14" t="s">
-        <v>101</v>
+      <c r="F43" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="G43" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="H43" s="12" t="s">
+        <v>115</v>
       </c>
       <c r="I43" s="14" t="s">
         <v>126</v>
@@ -2379,30 +2379,30 @@
         <v>143</v>
       </c>
     </row>
-    <row r="44" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A44" s="14">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B44" s="3" t="s">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>103</v>
-      </c>
-      <c r="D44" s="12">
-        <v>1.36</v>
+        <v>91</v>
+      </c>
+      <c r="D44" s="14">
+        <v>0.33</v>
       </c>
       <c r="E44" s="14" t="s">
         <v>156</v>
       </c>
       <c r="F44" s="14">
-        <v>304</v>
+        <v>4.7649999999999997</v>
       </c>
       <c r="G44" s="14">
-        <v>4920</v>
+        <v>2299</v>
       </c>
       <c r="H44" s="14" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="I44" s="14" t="s">
         <v>126</v>
@@ -2411,30 +2411,30 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A45" s="14">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="B45" s="3" t="s">
-        <v>104</v>
+        <v>18</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>105</v>
+        <v>19</v>
       </c>
       <c r="D45" s="14">
-        <v>1.962</v>
+        <v>8.48</v>
       </c>
       <c r="E45" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F45" s="12">
-        <v>2153</v>
-      </c>
-      <c r="G45" s="12">
-        <v>38120</v>
-      </c>
-      <c r="H45" s="12" t="s">
-        <v>146</v>
+      <c r="F45" s="14">
+        <v>158</v>
+      </c>
+      <c r="G45" s="14">
+        <v>2844</v>
+      </c>
+      <c r="H45" s="14" t="s">
+        <v>20</v>
       </c>
       <c r="I45" s="14" t="s">
         <v>126</v>
@@ -2443,30 +2443,30 @@
         <v>147</v>
       </c>
     </row>
-    <row r="46" spans="1:10" ht="46.8" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A46" s="14">
-        <v>45</v>
-      </c>
-      <c r="B46" s="5" t="s">
-        <v>106</v>
+        <v>39</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>92</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="D46" s="17">
-        <v>2.81</v>
+        <v>93</v>
+      </c>
+      <c r="D46" s="14">
+        <v>0.2</v>
       </c>
       <c r="E46" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F46" s="12">
-        <v>1636</v>
-      </c>
-      <c r="G46" s="12">
-        <v>1540</v>
-      </c>
-      <c r="H46" s="12" t="s">
-        <v>32</v>
+      <c r="F46" s="14">
+        <v>198</v>
+      </c>
+      <c r="G46" s="14">
+        <v>721</v>
+      </c>
+      <c r="H46" s="14" t="s">
+        <v>141</v>
       </c>
       <c r="I46" s="14" t="s">
         <v>126</v>
@@ -2475,60 +2475,60 @@
         <v>148</v>
       </c>
     </row>
-    <row r="47" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A47" s="14">
-        <v>46</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>110</v>
+        <v>44</v>
+      </c>
+      <c r="B47" s="3" t="s">
+        <v>104</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>108</v>
-      </c>
-      <c r="D47" s="5">
-        <v>844.91</v>
+        <v>105</v>
+      </c>
+      <c r="D47" s="14">
+        <v>1.962</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>155</v>
-      </c>
-      <c r="F47" s="18">
-        <v>2233</v>
-      </c>
-      <c r="G47" s="18">
-        <v>12655</v>
-      </c>
-      <c r="H47" s="5" t="s">
-        <v>76</v>
+        <v>156</v>
+      </c>
+      <c r="F47" s="12">
+        <v>2153</v>
+      </c>
+      <c r="G47" s="12">
+        <v>38120</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>146</v>
       </c>
       <c r="I47" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J47" s="12"/>
     </row>
-    <row r="48" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A48" s="14">
+        <v>21</v>
+      </c>
+      <c r="B48" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="C48" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="D48" s="14">
+        <v>2.63</v>
+      </c>
+      <c r="E48" s="14" t="s">
+        <v>156</v>
+      </c>
+      <c r="F48" s="14">
+        <v>12821</v>
+      </c>
+      <c r="G48" s="14">
+        <v>140</v>
+      </c>
+      <c r="H48" s="14" t="s">
         <v>47</v>
-      </c>
-      <c r="B48" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="C48" s="5" t="s">
-        <v>123</v>
-      </c>
-      <c r="D48" s="5">
-        <v>0.37</v>
-      </c>
-      <c r="E48" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F48" s="5">
-        <v>653</v>
-      </c>
-      <c r="G48" s="18">
-        <v>6249</v>
-      </c>
-      <c r="H48" s="5" t="s">
-        <v>109</v>
       </c>
       <c r="I48" s="14" t="s">
         <v>126</v>
@@ -2537,30 +2537,30 @@
         <v>150</v>
       </c>
     </row>
-    <row r="49" spans="1:10" ht="18.600000000000001" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A49" s="14">
-        <v>48</v>
-      </c>
-      <c r="B49" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="D49" s="12">
-        <v>3.2000000000000001E-2</v>
+        <v>29</v>
+      </c>
+      <c r="B49" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="D49" s="14">
+        <v>25000</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F49" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="G49" s="12">
-        <v>425</v>
-      </c>
-      <c r="H49" s="12" t="s">
-        <v>115</v>
+        <v>155</v>
+      </c>
+      <c r="F49" s="14">
+        <v>1134</v>
+      </c>
+      <c r="G49" s="14">
+        <v>369</v>
+      </c>
+      <c r="H49" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="I49" s="14" t="s">
         <v>126</v>
@@ -2569,60 +2569,60 @@
         <v>151</v>
       </c>
     </row>
-    <row r="50" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A50" s="14">
-        <v>49</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C50" s="12" t="s">
-        <v>119</v>
+        <v>43</v>
+      </c>
+      <c r="B50" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="C50" s="5" t="s">
+        <v>103</v>
       </c>
       <c r="D50" s="12">
-        <v>0.95799999999999996</v>
+        <v>1.36</v>
       </c>
       <c r="E50" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F50" s="12">
-        <v>1652</v>
-      </c>
-      <c r="G50" s="12">
-        <v>1972</v>
-      </c>
-      <c r="H50" s="12" t="s">
-        <v>32</v>
+      <c r="F50" s="14">
+        <v>304</v>
+      </c>
+      <c r="G50" s="14">
+        <v>4920</v>
+      </c>
+      <c r="H50" s="14" t="s">
+        <v>144</v>
       </c>
       <c r="I50" s="14" t="s">
         <v>126</v>
       </c>
       <c r="J50" s="12"/>
     </row>
-    <row r="51" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:10" ht="18.75" x14ac:dyDescent="0.25">
       <c r="A51" s="14">
+        <v>31</v>
+      </c>
+      <c r="B51" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="D51" s="16">
+        <v>1545</v>
+      </c>
+      <c r="E51" s="14" t="s">
+        <v>155</v>
+      </c>
+      <c r="F51" s="16">
+        <v>262</v>
+      </c>
+      <c r="G51" s="16">
         <v>50</v>
       </c>
-      <c r="B51" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="C51" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="D51" s="12">
-        <v>1.2</v>
-      </c>
-      <c r="E51" s="14" t="s">
-        <v>156</v>
-      </c>
-      <c r="F51" s="12">
-        <v>2153</v>
-      </c>
-      <c r="G51" s="13">
-        <v>38120</v>
-      </c>
-      <c r="H51" s="12" t="s">
-        <v>146</v>
+      <c r="H51" s="16" t="s">
+        <v>76</v>
       </c>
       <c r="I51" s="14" t="s">
         <v>126</v>
@@ -2631,55 +2631,55 @@
         <v>152</v>
       </c>
     </row>
-    <row r="52" spans="1:10" ht="31.2" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:10" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A52" s="14">
-        <v>51</v>
-      </c>
-      <c r="B52" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="C52" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="D52" s="12">
-        <v>6.2E-2</v>
+        <v>32</v>
+      </c>
+      <c r="B52" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="D52" s="14">
+        <v>0.7</v>
       </c>
       <c r="E52" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="F52" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="G52" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="H52" s="12" t="s">
-        <v>115</v>
+      <c r="F52" s="14">
+        <v>844</v>
+      </c>
+      <c r="G52" s="14">
+        <v>12872</v>
+      </c>
+      <c r="H52" s="14" t="s">
+        <v>79</v>
       </c>
       <c r="I52" s="12"/>
       <c r="J52" s="12" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A53" s="2"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A54" s="2"/>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A55" s="2"/>
       <c r="B55" s="7"/>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A56" s="2"/>
       <c r="B56" s="7"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A57" s="2"/>
       <c r="B57" s="7"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A58" s="2"/>
       <c r="C58" s="4"/>
       <c r="D58" s="2"/>
@@ -2689,7 +2689,7 @@
       <c r="H58" s="2"/>
       <c r="I58" s="2"/>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A59" s="2"/>
       <c r="C59" s="4"/>
       <c r="D59" s="2"/>
@@ -2699,7 +2699,7 @@
       <c r="H59" s="2"/>
       <c r="I59" s="2"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A60" s="2"/>
       <c r="C60" s="4"/>
       <c r="D60" s="2"/>
@@ -2709,7 +2709,7 @@
       <c r="H60" s="2"/>
       <c r="I60" s="2"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A61" s="2"/>
       <c r="C61" s="4"/>
       <c r="D61" s="2"/>
@@ -2719,7 +2719,7 @@
       <c r="H61" s="2"/>
       <c r="I61" s="2"/>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A62" s="2"/>
       <c r="C62" s="4"/>
       <c r="D62" s="2"/>
@@ -2729,7 +2729,7 @@
       <c r="H62" s="2"/>
       <c r="I62" s="2"/>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A63" s="2"/>
       <c r="C63" s="6"/>
       <c r="D63" s="6"/>
@@ -2739,7 +2739,7 @@
       <c r="H63" s="6"/>
       <c r="I63" s="6"/>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A64" s="2"/>
       <c r="C64" s="4"/>
       <c r="D64" s="2"/>
@@ -2749,7 +2749,7 @@
       <c r="H64" s="2"/>
       <c r="I64" s="2"/>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>
       <c r="C65" s="4"/>
       <c r="D65" s="2"/>
@@ -2759,7 +2759,7 @@
       <c r="H65" s="2"/>
       <c r="I65" s="2"/>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A66" s="2"/>
       <c r="C66" s="6"/>
       <c r="D66" s="6"/>
@@ -2769,7 +2769,7 @@
       <c r="H66" s="6"/>
       <c r="I66" s="6"/>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A67" s="2"/>
       <c r="C67" s="6"/>
       <c r="D67" s="6"/>
@@ -2779,19 +2779,19 @@
       <c r="H67" s="6"/>
       <c r="I67" s="6"/>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A68" s="2"/>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A69" s="2"/>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A70" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:H67" xr:uid="{9EE16F5C-9A23-431F-BBFB-BA5A34AA640B}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:J52">
-      <sortCondition ref="A1:A67"/>
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:H67">
+      <sortCondition ref="B1:B67"/>
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>